<commit_message>
Standardize Census names Chhachhundra to छछून्दरा and Ghana to घणा across master data; organize pending syllabus files into dedicated folder
</commit_message>
<xml_diff>
--- a/school enrolment.xlsx
+++ b/school enrolment.xlsx
@@ -3361,7 +3361,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>रा.उ.मा.वि. छाछून्दरा (GOVT. SENIOR SECONDARY SCHOOL CHHACHHUNDRA)</t>
+          <t>रा.उ.मा.वि. छछून्दरा (GOVT. SENIOR SECONDARY SCHOOL CHHACHHUNDRA)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>रा.उ.मा.वि. घाणा (GOVT. SENIOR SECONDARY SCHOOL GHANA)</t>
+          <t>रा.उ.मा.वि. घणा (GOVT. SENIOR SECONDARY SCHOOL GHANA)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">

</xml_diff>